<commit_message>
Envelope processing done correctly
</commit_message>
<xml_diff>
--- a/wwwroot/142/CatchSummary.xlsx
+++ b/wwwroot/142/CatchSummary.xlsx
@@ -476,7 +476,7 @@
         <v>5</v>
       </c>
       <c r="B2" s="0">
-        <v>0</v>
+        <v>1070</v>
       </c>
       <c r="C2" s="0">
         <v>107</v>
@@ -493,7 +493,7 @@
         <v>6</v>
       </c>
       <c r="B3" s="0">
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="C3" s="0">
         <v>90</v>
@@ -510,7 +510,7 @@
         <v>7</v>
       </c>
       <c r="B4" s="0">
-        <v>0</v>
+        <v>990</v>
       </c>
       <c r="C4" s="0">
         <v>99</v>
@@ -527,7 +527,7 @@
         <v>8</v>
       </c>
       <c r="B5" s="0">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="C5" s="0">
         <v>500</v>
@@ -544,7 +544,7 @@
         <v>9</v>
       </c>
       <c r="B6" s="0">
-        <v>0</v>
+        <v>1380</v>
       </c>
       <c r="C6" s="0">
         <v>138</v>
@@ -561,7 +561,7 @@
         <v>10</v>
       </c>
       <c r="B7" s="0">
-        <v>0</v>
+        <v>1040</v>
       </c>
       <c r="C7" s="0">
         <v>104</v>
@@ -578,7 +578,7 @@
         <v>11</v>
       </c>
       <c r="B8" s="0">
-        <v>0</v>
+        <v>1170</v>
       </c>
       <c r="C8" s="0">
         <v>117</v>
@@ -595,7 +595,7 @@
         <v>12</v>
       </c>
       <c r="B9" s="0">
-        <v>0</v>
+        <v>1150</v>
       </c>
       <c r="C9" s="0">
         <v>115</v>
@@ -612,7 +612,7 @@
         <v>13</v>
       </c>
       <c r="B10" s="0">
-        <v>0</v>
+        <v>840</v>
       </c>
       <c r="C10" s="0">
         <v>84</v>
@@ -629,7 +629,7 @@
         <v>14</v>
       </c>
       <c r="B11" s="0">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="C11" s="0">
         <v>64</v>
@@ -646,7 +646,7 @@
         <v>15</v>
       </c>
       <c r="B12" s="0">
-        <v>0</v>
+        <v>3820</v>
       </c>
       <c r="C12" s="0">
         <v>382</v>
@@ -663,7 +663,7 @@
         <v>16</v>
       </c>
       <c r="B13" s="0">
-        <v>0</v>
+        <v>2090</v>
       </c>
       <c r="C13" s="0">
         <v>209</v>
@@ -680,7 +680,7 @@
         <v>17</v>
       </c>
       <c r="B14" s="0">
-        <v>0</v>
+        <v>950</v>
       </c>
       <c r="C14" s="0">
         <v>95</v>
@@ -697,7 +697,7 @@
         <v>18</v>
       </c>
       <c r="B15" s="0">
-        <v>0</v>
+        <v>2140</v>
       </c>
       <c r="C15" s="0">
         <v>214</v>
@@ -714,7 +714,7 @@
         <v>19</v>
       </c>
       <c r="B16" s="0">
-        <v>0</v>
+        <v>1660</v>
       </c>
       <c r="C16" s="0">
         <v>166</v>
@@ -731,7 +731,7 @@
         <v>20</v>
       </c>
       <c r="B17" s="0">
-        <v>0</v>
+        <v>1390</v>
       </c>
       <c r="C17" s="0">
         <v>139</v>
@@ -748,7 +748,7 @@
         <v>21</v>
       </c>
       <c r="B18" s="0">
-        <v>0</v>
+        <v>1020</v>
       </c>
       <c r="C18" s="0">
         <v>102</v>
@@ -765,7 +765,7 @@
         <v>22</v>
       </c>
       <c r="B19" s="0">
-        <v>0</v>
+        <v>1120</v>
       </c>
       <c r="C19" s="0">
         <v>112</v>
@@ -782,7 +782,7 @@
         <v>23</v>
       </c>
       <c r="B20" s="0">
-        <v>0</v>
+        <v>810</v>
       </c>
       <c r="C20" s="0">
         <v>81</v>
@@ -799,7 +799,7 @@
         <v>24</v>
       </c>
       <c r="B21" s="0">
-        <v>0</v>
+        <v>3790</v>
       </c>
       <c r="C21" s="0">
         <v>379</v>
@@ -816,7 +816,7 @@
         <v>25</v>
       </c>
       <c r="B22" s="0">
-        <v>0</v>
+        <v>1070</v>
       </c>
       <c r="C22" s="0">
         <v>107</v>
@@ -833,7 +833,7 @@
         <v>26</v>
       </c>
       <c r="B23" s="0">
-        <v>0</v>
+        <v>3850</v>
       </c>
       <c r="C23" s="0">
         <v>385</v>
@@ -850,7 +850,7 @@
         <v>27</v>
       </c>
       <c r="B24" s="0">
-        <v>0</v>
+        <v>1710</v>
       </c>
       <c r="C24" s="0">
         <v>171</v>
@@ -867,7 +867,7 @@
         <v>28</v>
       </c>
       <c r="B25" s="0">
-        <v>0</v>
+        <v>1870</v>
       </c>
       <c r="C25" s="0">
         <v>187</v>
@@ -884,7 +884,7 @@
         <v>29</v>
       </c>
       <c r="B26" s="0">
-        <v>0</v>
+        <v>2060</v>
       </c>
       <c r="C26" s="0">
         <v>206</v>
@@ -901,7 +901,7 @@
         <v>30</v>
       </c>
       <c r="B27" s="0">
-        <v>0</v>
+        <v>1560</v>
       </c>
       <c r="C27" s="0">
         <v>156</v>
@@ -918,7 +918,7 @@
         <v>31</v>
       </c>
       <c r="B28" s="0">
-        <v>0</v>
+        <v>1490</v>
       </c>
       <c r="C28" s="0">
         <v>149</v>
@@ -935,7 +935,7 @@
         <v>32</v>
       </c>
       <c r="B29" s="0">
-        <v>0</v>
+        <v>1900</v>
       </c>
       <c r="C29" s="0">
         <v>190</v>
@@ -952,7 +952,7 @@
         <v>33</v>
       </c>
       <c r="B30" s="0">
-        <v>0</v>
+        <v>780</v>
       </c>
       <c r="C30" s="0">
         <v>78</v>
@@ -969,7 +969,7 @@
         <v>34</v>
       </c>
       <c r="B31" s="0">
-        <v>0</v>
+        <v>270</v>
       </c>
       <c r="C31" s="0">
         <v>27</v>
@@ -986,7 +986,7 @@
         <v>35</v>
       </c>
       <c r="B32" s="0">
-        <v>0</v>
+        <v>2600</v>
       </c>
       <c r="C32" s="0">
         <v>260</v>
@@ -1003,7 +1003,7 @@
         <v>36</v>
       </c>
       <c r="B33" s="0">
-        <v>0</v>
+        <v>3540</v>
       </c>
       <c r="C33" s="0">
         <v>354</v>
@@ -1020,7 +1020,7 @@
         <v>37</v>
       </c>
       <c r="B34" s="0">
-        <v>0</v>
+        <v>1480</v>
       </c>
       <c r="C34" s="0">
         <v>148</v>
@@ -1037,7 +1037,7 @@
         <v>38</v>
       </c>
       <c r="B35" s="0">
-        <v>0</v>
+        <v>1710</v>
       </c>
       <c r="C35" s="0">
         <v>171</v>
@@ -1054,7 +1054,7 @@
         <v>39</v>
       </c>
       <c r="B36" s="0">
-        <v>0</v>
+        <v>570</v>
       </c>
       <c r="C36" s="0">
         <v>57</v>
@@ -1071,7 +1071,7 @@
         <v>40</v>
       </c>
       <c r="B37" s="0">
-        <v>0</v>
+        <v>1870</v>
       </c>
       <c r="C37" s="0">
         <v>187</v>
@@ -1088,7 +1088,7 @@
         <v>41</v>
       </c>
       <c r="B38" s="0">
-        <v>0</v>
+        <v>2080</v>
       </c>
       <c r="C38" s="0">
         <v>208</v>
@@ -1105,7 +1105,7 @@
         <v>42</v>
       </c>
       <c r="B39" s="0">
-        <v>0</v>
+        <v>1580</v>
       </c>
       <c r="C39" s="0">
         <v>158</v>
@@ -1122,7 +1122,7 @@
         <v>43</v>
       </c>
       <c r="B40" s="0">
-        <v>0</v>
+        <v>1470</v>
       </c>
       <c r="C40" s="0">
         <v>147</v>
@@ -1139,7 +1139,7 @@
         <v>44</v>
       </c>
       <c r="B41" s="0">
-        <v>0</v>
+        <v>1890</v>
       </c>
       <c r="C41" s="0">
         <v>189</v>
@@ -1156,7 +1156,7 @@
         <v>45</v>
       </c>
       <c r="B42" s="0">
-        <v>0</v>
+        <v>810</v>
       </c>
       <c r="C42" s="0">
         <v>81</v>
@@ -1173,7 +1173,7 @@
         <v>46</v>
       </c>
       <c r="B43" s="0">
-        <v>0</v>
+        <v>540</v>
       </c>
       <c r="C43" s="0">
         <v>54</v>
@@ -1190,7 +1190,7 @@
         <v>47</v>
       </c>
       <c r="B44" s="0">
-        <v>0</v>
+        <v>2770</v>
       </c>
       <c r="C44" s="0">
         <v>277</v>
@@ -1207,7 +1207,7 @@
         <v>48</v>
       </c>
       <c r="B45" s="0">
-        <v>0</v>
+        <v>2640</v>
       </c>
       <c r="C45" s="0">
         <v>264</v>
@@ -1224,7 +1224,7 @@
         <v>49</v>
       </c>
       <c r="B46" s="0">
-        <v>0</v>
+        <v>1100</v>
       </c>
       <c r="C46" s="0">
         <v>110</v>
@@ -1241,7 +1241,7 @@
         <v>50</v>
       </c>
       <c r="B47" s="0">
-        <v>0</v>
+        <v>1690</v>
       </c>
       <c r="C47" s="0">
         <v>169</v>
@@ -1258,7 +1258,7 @@
         <v>51</v>
       </c>
       <c r="B48" s="0">
-        <v>0</v>
+        <v>560</v>
       </c>
       <c r="C48" s="0">
         <v>56</v>
@@ -1275,7 +1275,7 @@
         <v>52</v>
       </c>
       <c r="B49" s="0">
-        <v>0</v>
+        <v>1700</v>
       </c>
       <c r="C49" s="0">
         <v>170</v>
@@ -1292,7 +1292,7 @@
         <v>53</v>
       </c>
       <c r="B50" s="0">
-        <v>0</v>
+        <v>1960</v>
       </c>
       <c r="C50" s="0">
         <v>196</v>
@@ -1309,7 +1309,7 @@
         <v>54</v>
       </c>
       <c r="B51" s="0">
-        <v>0</v>
+        <v>1530</v>
       </c>
       <c r="C51" s="0">
         <v>153</v>
@@ -1326,7 +1326,7 @@
         <v>55</v>
       </c>
       <c r="B52" s="0">
-        <v>0</v>
+        <v>1420</v>
       </c>
       <c r="C52" s="0">
         <v>142</v>
@@ -1343,7 +1343,7 @@
         <v>56</v>
       </c>
       <c r="B53" s="0">
-        <v>0</v>
+        <v>1820</v>
       </c>
       <c r="C53" s="0">
         <v>182</v>
@@ -1360,7 +1360,7 @@
         <v>57</v>
       </c>
       <c r="B54" s="0">
-        <v>0</v>
+        <v>780</v>
       </c>
       <c r="C54" s="0">
         <v>78</v>
@@ -1377,7 +1377,7 @@
         <v>58</v>
       </c>
       <c r="B55" s="0">
-        <v>0</v>
+        <v>480</v>
       </c>
       <c r="C55" s="0">
         <v>48</v>
@@ -1394,7 +1394,7 @@
         <v>59</v>
       </c>
       <c r="B56" s="0">
-        <v>0</v>
+        <v>2700</v>
       </c>
       <c r="C56" s="0">
         <v>270</v>
@@ -1411,7 +1411,7 @@
         <v>60</v>
       </c>
       <c r="B57" s="0">
-        <v>0</v>
+        <v>1040</v>
       </c>
       <c r="C57" s="0">
         <v>104</v>
@@ -1428,7 +1428,7 @@
         <v>61</v>
       </c>
       <c r="B58" s="0">
-        <v>0</v>
+        <v>450</v>
       </c>
       <c r="C58" s="0">
         <v>45</v>
@@ -1445,7 +1445,7 @@
         <v>62</v>
       </c>
       <c r="B59" s="0">
-        <v>0</v>
+        <v>1690</v>
       </c>
       <c r="C59" s="0">
         <v>169</v>
@@ -1462,7 +1462,7 @@
         <v>63</v>
       </c>
       <c r="B60" s="0">
-        <v>0</v>
+        <v>1950</v>
       </c>
       <c r="C60" s="0">
         <v>195</v>
@@ -1479,7 +1479,7 @@
         <v>64</v>
       </c>
       <c r="B61" s="0">
-        <v>0</v>
+        <v>1410</v>
       </c>
       <c r="C61" s="0">
         <v>141</v>
@@ -1496,7 +1496,7 @@
         <v>65</v>
       </c>
       <c r="B62" s="0">
-        <v>0</v>
+        <v>1820</v>
       </c>
       <c r="C62" s="0">
         <v>182</v>
@@ -1513,7 +1513,7 @@
         <v>66</v>
       </c>
       <c r="B63" s="0">
-        <v>0</v>
+        <v>780</v>
       </c>
       <c r="C63" s="0">
         <v>78</v>
@@ -1530,7 +1530,7 @@
         <v>67</v>
       </c>
       <c r="B64" s="0">
-        <v>0</v>
+        <v>2010</v>
       </c>
       <c r="C64" s="0">
         <v>201</v>
@@ -1547,7 +1547,7 @@
         <v>68</v>
       </c>
       <c r="B65" s="0">
-        <v>0</v>
+        <v>1940</v>
       </c>
       <c r="C65" s="0">
         <v>194</v>
@@ -1564,7 +1564,7 @@
         <v>69</v>
       </c>
       <c r="B66" s="0">
-        <v>0</v>
+        <v>2070</v>
       </c>
       <c r="C66" s="0">
         <v>207</v>
@@ -1581,7 +1581,7 @@
         <v>70</v>
       </c>
       <c r="B67" s="0">
-        <v>0</v>
+        <v>1300</v>
       </c>
       <c r="C67" s="0">
         <v>130</v>
@@ -1598,7 +1598,7 @@
         <v>71</v>
       </c>
       <c r="B68" s="0">
-        <v>0</v>
+        <v>2870</v>
       </c>
       <c r="C68" s="0">
         <v>287</v>
@@ -1615,7 +1615,7 @@
         <v>72</v>
       </c>
       <c r="B69" s="0">
-        <v>0</v>
+        <v>1570</v>
       </c>
       <c r="C69" s="0">
         <v>157</v>
@@ -1632,7 +1632,7 @@
         <v>73</v>
       </c>
       <c r="B70" s="0">
-        <v>0</v>
+        <v>990</v>
       </c>
       <c r="C70" s="0">
         <v>99</v>
@@ -1649,7 +1649,7 @@
         <v>74</v>
       </c>
       <c r="B71" s="0">
-        <v>0</v>
+        <v>1160</v>
       </c>
       <c r="C71" s="0">
         <v>116</v>
@@ -1666,7 +1666,7 @@
         <v>75</v>
       </c>
       <c r="B72" s="0">
-        <v>0</v>
+        <v>1020</v>
       </c>
       <c r="C72" s="0">
         <v>102</v>
@@ -1683,7 +1683,7 @@
         <v>76</v>
       </c>
       <c r="B73" s="0">
-        <v>0</v>
+        <v>1160</v>
       </c>
       <c r="C73" s="0">
         <v>116</v>
@@ -1700,7 +1700,7 @@
         <v>77</v>
       </c>
       <c r="B74" s="0">
-        <v>0</v>
+        <v>1080</v>
       </c>
       <c r="C74" s="0">
         <v>108</v>
@@ -1717,7 +1717,7 @@
         <v>78</v>
       </c>
       <c r="B75" s="0">
-        <v>0</v>
+        <v>2030</v>
       </c>
       <c r="C75" s="0">
         <v>203</v>
@@ -1734,7 +1734,7 @@
         <v>79</v>
       </c>
       <c r="B76" s="0">
-        <v>0</v>
+        <v>1050</v>
       </c>
       <c r="C76" s="0">
         <v>105</v>
@@ -1751,7 +1751,7 @@
         <v>80</v>
       </c>
       <c r="B77" s="0">
-        <v>0</v>
+        <v>1300</v>
       </c>
       <c r="C77" s="0">
         <v>130</v>
@@ -1768,7 +1768,7 @@
         <v>81</v>
       </c>
       <c r="B78" s="0">
-        <v>0</v>
+        <v>990</v>
       </c>
       <c r="C78" s="0">
         <v>99</v>
@@ -1785,7 +1785,7 @@
         <v>82</v>
       </c>
       <c r="B79" s="0">
-        <v>0</v>
+        <v>1160</v>
       </c>
       <c r="C79" s="0">
         <v>116</v>
@@ -1802,7 +1802,7 @@
         <v>83</v>
       </c>
       <c r="B80" s="0">
-        <v>0</v>
+        <v>1010</v>
       </c>
       <c r="C80" s="0">
         <v>101</v>
@@ -1819,7 +1819,7 @@
         <v>84</v>
       </c>
       <c r="B81" s="0">
-        <v>0</v>
+        <v>1210</v>
       </c>
       <c r="C81" s="0">
         <v>121</v>
@@ -1836,7 +1836,7 @@
         <v>85</v>
       </c>
       <c r="B82" s="0">
-        <v>0</v>
+        <v>790</v>
       </c>
       <c r="C82" s="0">
         <v>79</v>
@@ -1853,7 +1853,7 @@
         <v>86</v>
       </c>
       <c r="B83" s="0">
-        <v>0</v>
+        <v>760</v>
       </c>
       <c r="C83" s="0">
         <v>76</v>
@@ -1870,7 +1870,7 @@
         <v>87</v>
       </c>
       <c r="B84" s="0">
-        <v>0</v>
+        <v>1600</v>
       </c>
       <c r="C84" s="0">
         <v>160</v>
@@ -1887,7 +1887,7 @@
         <v>88</v>
       </c>
       <c r="B85" s="0">
-        <v>0</v>
+        <v>1420</v>
       </c>
       <c r="C85" s="0">
         <v>142</v>
@@ -1904,7 +1904,7 @@
         <v>89</v>
       </c>
       <c r="B86" s="0">
-        <v>0</v>
+        <v>2090</v>
       </c>
       <c r="C86" s="0">
         <v>209</v>
@@ -1921,7 +1921,7 @@
         <v>90</v>
       </c>
       <c r="B87" s="0">
-        <v>0</v>
+        <v>1280</v>
       </c>
       <c r="C87" s="0">
         <v>128</v>
@@ -1938,7 +1938,7 @@
         <v>91</v>
       </c>
       <c r="B88" s="0">
-        <v>0</v>
+        <v>2420</v>
       </c>
       <c r="C88" s="0">
         <v>242</v>
@@ -1955,7 +1955,7 @@
         <v>92</v>
       </c>
       <c r="B89" s="0">
-        <v>0</v>
+        <v>1780</v>
       </c>
       <c r="C89" s="0">
         <v>178</v>
@@ -1972,7 +1972,7 @@
         <v>93</v>
       </c>
       <c r="B90" s="0">
-        <v>0</v>
+        <v>2050</v>
       </c>
       <c r="C90" s="0">
         <v>205</v>
@@ -1989,7 +1989,7 @@
         <v>94</v>
       </c>
       <c r="B91" s="0">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="C91" s="0">
         <v>100</v>
@@ -2006,7 +2006,7 @@
         <v>95</v>
       </c>
       <c r="B92" s="0">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="C92" s="0">
         <v>80</v>
@@ -2023,7 +2023,7 @@
         <v>96</v>
       </c>
       <c r="B93" s="0">
-        <v>0</v>
+        <v>1190</v>
       </c>
       <c r="C93" s="0">
         <v>119</v>
@@ -2040,7 +2040,7 @@
         <v>97</v>
       </c>
       <c r="B94" s="0">
-        <v>0</v>
+        <v>740</v>
       </c>
       <c r="C94" s="0">
         <v>74</v>
@@ -2057,7 +2057,7 @@
         <v>98</v>
       </c>
       <c r="B95" s="0">
-        <v>0</v>
+        <v>1470</v>
       </c>
       <c r="C95" s="0">
         <v>147</v>
@@ -2074,7 +2074,7 @@
         <v>99</v>
       </c>
       <c r="B96" s="0">
-        <v>0</v>
+        <v>3290</v>
       </c>
       <c r="C96" s="0">
         <v>329</v>
@@ -2091,7 +2091,7 @@
         <v>100</v>
       </c>
       <c r="B97" s="0">
-        <v>0</v>
+        <v>1270</v>
       </c>
       <c r="C97" s="0">
         <v>127</v>
@@ -2108,7 +2108,7 @@
         <v>101</v>
       </c>
       <c r="B98" s="0">
-        <v>0</v>
+        <v>1310</v>
       </c>
       <c r="C98" s="0">
         <v>131</v>
@@ -2125,7 +2125,7 @@
         <v>102</v>
       </c>
       <c r="B99" s="0">
-        <v>0</v>
+        <v>2420</v>
       </c>
       <c r="C99" s="0">
         <v>242</v>
@@ -2142,7 +2142,7 @@
         <v>103</v>
       </c>
       <c r="B100" s="0">
-        <v>0</v>
+        <v>1780</v>
       </c>
       <c r="C100" s="0">
         <v>178</v>
@@ -2159,7 +2159,7 @@
         <v>104</v>
       </c>
       <c r="B101" s="0">
-        <v>0</v>
+        <v>2040</v>
       </c>
       <c r="C101" s="0">
         <v>204</v>
@@ -2176,7 +2176,7 @@
         <v>105</v>
       </c>
       <c r="B102" s="0">
-        <v>0</v>
+        <v>990</v>
       </c>
       <c r="C102" s="0">
         <v>99</v>
@@ -2193,7 +2193,7 @@
         <v>106</v>
       </c>
       <c r="B103" s="0">
-        <v>0</v>
+        <v>860</v>
       </c>
       <c r="C103" s="0">
         <v>86</v>
@@ -2210,7 +2210,7 @@
         <v>107</v>
       </c>
       <c r="B104" s="0">
-        <v>0</v>
+        <v>1210</v>
       </c>
       <c r="C104" s="0">
         <v>121</v>
@@ -2227,7 +2227,7 @@
         <v>108</v>
       </c>
       <c r="B105" s="0">
-        <v>0</v>
+        <v>770</v>
       </c>
       <c r="C105" s="0">
         <v>77</v>
@@ -2244,7 +2244,7 @@
         <v>109</v>
       </c>
       <c r="B106" s="0">
-        <v>0</v>
+        <v>3160</v>
       </c>
       <c r="C106" s="0">
         <v>316</v>
@@ -2261,7 +2261,7 @@
         <v>110</v>
       </c>
       <c r="B107" s="0">
-        <v>0</v>
+        <v>1720</v>
       </c>
       <c r="C107" s="0">
         <v>172</v>
@@ -2278,7 +2278,7 @@
         <v>111</v>
       </c>
       <c r="B108" s="0">
-        <v>0</v>
+        <v>3020</v>
       </c>
       <c r="C108" s="0">
         <v>302</v>
@@ -2295,7 +2295,7 @@
         <v>112</v>
       </c>
       <c r="B109" s="0">
-        <v>0</v>
+        <v>1380</v>
       </c>
       <c r="C109" s="0">
         <v>138</v>
@@ -2312,7 +2312,7 @@
         <v>113</v>
       </c>
       <c r="B110" s="0">
-        <v>0</v>
+        <v>2300</v>
       </c>
       <c r="C110" s="0">
         <v>230</v>
@@ -2329,7 +2329,7 @@
         <v>114</v>
       </c>
       <c r="B111" s="0">
-        <v>0</v>
+        <v>1730</v>
       </c>
       <c r="C111" s="0">
         <v>173</v>
@@ -2346,7 +2346,7 @@
         <v>115</v>
       </c>
       <c r="B112" s="0">
-        <v>0</v>
+        <v>1940</v>
       </c>
       <c r="C112" s="0">
         <v>194</v>
@@ -2363,7 +2363,7 @@
         <v>116</v>
       </c>
       <c r="B113" s="0">
-        <v>0</v>
+        <v>990</v>
       </c>
       <c r="C113" s="0">
         <v>99</v>
@@ -2380,7 +2380,7 @@
         <v>117</v>
       </c>
       <c r="B114" s="0">
-        <v>0</v>
+        <v>1210</v>
       </c>
       <c r="C114" s="0">
         <v>121</v>
@@ -2397,7 +2397,7 @@
         <v>118</v>
       </c>
       <c r="B115" s="0">
-        <v>0</v>
+        <v>3330</v>
       </c>
       <c r="C115" s="0">
         <v>333</v>
@@ -2414,7 +2414,7 @@
         <v>119</v>
       </c>
       <c r="B116" s="0">
-        <v>0</v>
+        <v>1570</v>
       </c>
       <c r="C116" s="0">
         <v>157</v>
@@ -2431,7 +2431,7 @@
         <v>120</v>
       </c>
       <c r="B117" s="0">
-        <v>0</v>
+        <v>2400</v>
       </c>
       <c r="C117" s="0">
         <v>240</v>
@@ -2448,7 +2448,7 @@
         <v>121</v>
       </c>
       <c r="B118" s="0">
-        <v>0</v>
+        <v>1780</v>
       </c>
       <c r="C118" s="0">
         <v>178</v>
@@ -2465,7 +2465,7 @@
         <v>122</v>
       </c>
       <c r="B119" s="0">
-        <v>0</v>
+        <v>2040</v>
       </c>
       <c r="C119" s="0">
         <v>204</v>
@@ -2482,7 +2482,7 @@
         <v>123</v>
       </c>
       <c r="B120" s="0">
-        <v>0</v>
+        <v>990</v>
       </c>
       <c r="C120" s="0">
         <v>99</v>
@@ -2499,7 +2499,7 @@
         <v>124</v>
       </c>
       <c r="B121" s="0">
-        <v>0</v>
+        <v>810</v>
       </c>
       <c r="C121" s="0">
         <v>81</v>
@@ -2516,7 +2516,7 @@
         <v>125</v>
       </c>
       <c r="B122" s="0">
-        <v>0</v>
+        <v>730</v>
       </c>
       <c r="C122" s="0">
         <v>73</v>
@@ -2533,7 +2533,7 @@
         <v>126</v>
       </c>
       <c r="B123" s="0">
-        <v>0</v>
+        <v>480</v>
       </c>
       <c r="C123" s="0">
         <v>48</v>

</xml_diff>